<commit_message>
Fix template test portability and layout
</commit_message>
<xml_diff>
--- a/examples/示例资料库.xlsx
+++ b/examples/示例资料库.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R8faaaf6bf12246d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="个人资料" sheetId="2" r:id="Rd50793b9c242436a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经历清单" sheetId="3" r:id="R3c38aba50d544540"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="附件清单" sheetId="4" r:id="Ra1e53c04dadf4350"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R774fafdde7ef4b92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="个人资料" sheetId="2" r:id="R7d2c180b017f4d04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经历清单" sheetId="3" r:id="Re53c0dbf0bcc4e43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="附件清单" sheetId="4" r:id="Rc84383ee71ee464a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -652,7 +652,7 @@
   <x:cols>
     <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="32" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>

</xml_diff>

<commit_message>
test: checkpoint regenerated template artifacts
</commit_message>
<xml_diff>
--- a/examples/示例资料库.xlsx
+++ b/examples/示例资料库.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R774fafdde7ef4b92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="个人资料" sheetId="2" r:id="R7d2c180b017f4d04"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经历清单" sheetId="3" r:id="Re53c0dbf0bcc4e43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="附件清单" sheetId="4" r:id="Rc84383ee71ee464a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R6928d2ae7cc048af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="个人资料" sheetId="2" r:id="R4dfed2f2a84046b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经历清单" sheetId="3" r:id="R490dc603fa14412b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="附件清单" sheetId="4" r:id="Rcd4ab4c0e7a34009"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Fix profile validator aliases and date identities
</commit_message>
<xml_diff>
--- a/examples/示例资料库.xlsx
+++ b/examples/示例资料库.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R6928d2ae7cc048af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="个人资料" sheetId="2" r:id="R4dfed2f2a84046b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经历清单" sheetId="3" r:id="R490dc603fa14412b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="附件清单" sheetId="4" r:id="Rcd4ab4c0e7a34009"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R58f0d67430f6418f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="个人资料" sheetId="2" r:id="Rc0316d5ccc464ae9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经历清单" sheetId="3" r:id="R9c71c0f223ef4df2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="附件清单" sheetId="4" r:id="R75aa87a56a6e458c"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
docs: add local-only public skill guide
</commit_message>
<xml_diff>
--- a/examples/示例资料库.xlsx
+++ b/examples/示例资料库.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R58f0d67430f6418f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="个人资料" sheetId="2" r:id="Rc0316d5ccc464ae9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经历清单" sheetId="3" r:id="R9c71c0f223ef4df2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="附件清单" sheetId="4" r:id="R75aa87a56a6e458c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="Rd9da120cad994478"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="个人资料" sheetId="2" r:id="R6aee387a63e54ca2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经历清单" sheetId="3" r:id="Rad4bc1e5b7574195"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="附件清单" sheetId="4" r:id="R6ee5235c666040ab"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
test: isolate template generation outputs
</commit_message>
<xml_diff>
--- a/examples/示例资料库.xlsx
+++ b/examples/示例资料库.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R1ceee057f7ef479b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="个人资料" sheetId="2" r:id="R3a83064765284778"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经历清单" sheetId="3" r:id="Rc06c846780774a20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="附件清单" sheetId="4" r:id="R0612e8bfd90c4bb9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="Rdd35c032f52943b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="个人资料" sheetId="2" r:id="Red21213f01ca40bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经历清单" sheetId="3" r:id="Rc399a2244dd04372"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="附件清单" sheetId="4" r:id="R3c56f745aa564ada"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>